<commit_message>
change format template file
</commit_message>
<xml_diff>
--- a/frontend/public/templates/จัดการข้อมูล-ครูผู้สอน.xlsx
+++ b/frontend/public/templates/จัดการข้อมูล-ครูผู้สอน.xlsx
@@ -51,7 +51,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -62,6 +62,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFA64D79"/>
         <bgColor rgb="FFA64D79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +98,7 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>

</xml_diff>